<commit_message>
Update all 취합 aggregate Excel files with 19:00 최종 column on rightmost of every sheet
</commit_message>
<xml_diff>
--- a/web/public/2027대입_수시모집경쟁률취합_정보분석3팀_교대_최신.xlsx
+++ b/web/public/2027대입_수시모집경쟁률취합_정보분석3팀_교대_최신.xlsx
@@ -507,7 +507,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1641,7 +1641,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -2584,7 +2584,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -2971,7 +2971,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -3277,7 +3277,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -5359,7 +5359,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -6401,7 +6401,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -7075,7 +7075,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -9815,7 +9815,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -10121,7 +10121,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -10508,7 +10508,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S63"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -15123,7 +15123,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S56"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -19204,7 +19204,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -20055,7 +20055,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -20442,7 +20442,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -21385,7 +21385,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24040,7 +24040,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Fix 1-column shift in aggregate Excel by aligning 2 fixed columns with time series start at column C
</commit_message>
<xml_diff>
--- a/web/public/2027대입_수시모집경쟁률취합_정보분석3팀_교대_최신.xlsx
+++ b/web/public/2027대입_수시모집경쟁률취합_정보분석3팀_교대_최신.xlsx
@@ -506,28 +506,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,57 +535,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -702,7 +702,7 @@
           <t>402</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>326</t>
         </is>
@@ -893,7 +893,7 @@
           <t>110</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>54</t>
         </is>
@@ -985,7 +985,7 @@
           <t>226</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>209</t>
         </is>
@@ -1077,7 +1077,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1169,7 +1169,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -1261,7 +1261,7 @@
           <t>21</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -1353,7 +1353,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -1445,7 +1445,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -1537,7 +1537,7 @@
           <t>402</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>326</t>
         </is>
@@ -1620,15 +1620,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1640,28 +1640,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1670,57 +1669,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -1836,7 +1836,7 @@
           <t>96</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>105</t>
         </is>
@@ -1928,7 +1928,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -2020,7 +2020,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2112,7 +2112,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2204,7 +2204,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -2296,7 +2296,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -2388,7 +2388,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -2480,7 +2480,7 @@
           <t>184</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>166</t>
         </is>
@@ -2563,15 +2563,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2583,28 +2583,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2613,57 +2612,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -2779,7 +2779,7 @@
           <t>77</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
+      <c r="C5" s="8" t="inlineStr"/>
       <c r="D5" s="8" t="inlineStr"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
@@ -2839,7 +2839,7 @@
           <t>33</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
+      <c r="C6" s="8" t="inlineStr"/>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
@@ -2899,7 +2899,7 @@
           <t>110</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
@@ -2950,15 +2950,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2970,28 +2970,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3000,57 +2999,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -3173,7 +3173,7 @@
           <t>322</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>1,255</t>
         </is>
@@ -3256,15 +3256,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3276,28 +3276,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3306,57 +3305,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -3472,7 +3472,7 @@
           <t>315</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>503</t>
         </is>
@@ -3663,7 +3663,7 @@
           <t>220</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>398</t>
         </is>
@@ -3755,7 +3755,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>33</t>
         </is>
@@ -3847,7 +3847,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>44</t>
         </is>
@@ -3939,7 +3939,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -4031,7 +4031,7 @@
           <t>315</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>503</t>
         </is>
@@ -4222,7 +4222,7 @@
           <t>195</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>346</t>
         </is>
@@ -4314,7 +4314,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>52</t>
         </is>
@@ -4406,7 +4406,7 @@
           <t>220</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>398</t>
         </is>
@@ -4597,7 +4597,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>33</t>
         </is>
@@ -4689,7 +4689,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>33</t>
         </is>
@@ -4880,7 +4880,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>44</t>
         </is>
@@ -4972,7 +4972,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>44</t>
         </is>
@@ -5163,7 +5163,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -5255,7 +5255,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -5338,15 +5338,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5358,28 +5358,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5388,57 +5387,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -5554,7 +5554,7 @@
           <t>865</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>3,082</t>
         </is>
@@ -5745,7 +5745,7 @@
           <t>270</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>1,217</t>
         </is>
@@ -5837,7 +5837,7 @@
           <t>85</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>228</t>
         </is>
@@ -5929,7 +5929,7 @@
           <t>380</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>1,333</t>
         </is>
@@ -6021,7 +6021,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>155</t>
         </is>
@@ -6113,7 +6113,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>104</t>
         </is>
@@ -6205,7 +6205,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>45</t>
         </is>
@@ -6297,7 +6297,7 @@
           <t>865</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>3,082</t>
         </is>
@@ -6380,15 +6380,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6400,28 +6400,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6430,57 +6429,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -6596,7 +6596,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>290</t>
         </is>
@@ -6787,7 +6787,7 @@
           <t>90</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>265</t>
         </is>
@@ -6879,7 +6879,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -6971,7 +6971,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>290</t>
         </is>
@@ -7054,15 +7054,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7074,28 +7074,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7104,57 +7103,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -7270,7 +7270,7 @@
           <t>370</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>848</t>
         </is>
@@ -7461,7 +7461,7 @@
           <t>220</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>591</t>
         </is>
@@ -7553,7 +7553,7 @@
           <t>70</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>78</t>
         </is>
@@ -7645,7 +7645,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -7737,7 +7737,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -7829,7 +7829,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -7921,7 +7921,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>126</t>
         </is>
@@ -8013,7 +8013,7 @@
           <t>370</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>848</t>
         </is>
@@ -8204,7 +8204,7 @@
           <t>220</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>591</t>
         </is>
@@ -8296,7 +8296,7 @@
           <t>220</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>591</t>
         </is>
@@ -8487,7 +8487,7 @@
           <t>70</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>78</t>
         </is>
@@ -8579,7 +8579,7 @@
           <t>70</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>78</t>
         </is>
@@ -8770,7 +8770,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -8862,7 +8862,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -9053,7 +9053,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -9145,7 +9145,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -9336,7 +9336,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -9428,7 +9428,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -9619,7 +9619,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>126</t>
         </is>
@@ -9711,7 +9711,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>126</t>
         </is>
@@ -9794,15 +9794,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9814,28 +9814,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9844,57 +9843,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -10017,7 +10017,7 @@
           <t>565</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>1,736</t>
         </is>
@@ -10100,15 +10100,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10120,28 +10120,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10150,57 +10149,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -10316,7 +10316,7 @@
           <t>140</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
+      <c r="C5" s="8" t="inlineStr"/>
       <c r="D5" s="8" t="inlineStr"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
@@ -10376,7 +10376,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
+      <c r="C6" s="8" t="inlineStr"/>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
@@ -10436,7 +10436,7 @@
           <t>200</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
@@ -10487,15 +10487,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10507,28 +10507,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S63"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10537,57 +10536,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -10703,7 +10703,7 @@
           <t>272</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>211</t>
         </is>
@@ -10894,7 +10894,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -10986,7 +10986,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11078,7 +11078,7 @@
           <t>53</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>79</t>
         </is>
@@ -11170,7 +11170,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -11262,7 +11262,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -11354,7 +11354,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>35</t>
         </is>
@@ -11446,7 +11446,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -11538,7 +11538,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -11630,7 +11630,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -11722,7 +11722,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11814,7 +11814,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -11906,7 +11906,7 @@
           <t>272</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>211</t>
         </is>
@@ -12097,7 +12097,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -12189,7 +12189,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -12380,7 +12380,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -12472,7 +12472,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -12663,7 +12663,7 @@
           <t>53</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>79</t>
         </is>
@@ -12755,7 +12755,7 @@
           <t>53</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>79</t>
         </is>
@@ -12946,7 +12946,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -13038,7 +13038,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -13229,7 +13229,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -13321,7 +13321,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -13512,7 +13512,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>35</t>
         </is>
@@ -13604,7 +13604,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>35</t>
         </is>
@@ -13795,7 +13795,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -13887,7 +13887,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -14078,7 +14078,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -14170,7 +14170,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -14361,7 +14361,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C54" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -14453,7 +14453,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -14644,7 +14644,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="C58" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -14736,7 +14736,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -14927,7 +14927,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C62" s="7" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -15019,7 +15019,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -15102,15 +15102,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15123,21 +15123,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S56"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
@@ -15152,57 +15152,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -15318,7 +15319,7 @@
           <t>310</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>122</t>
         </is>
@@ -15509,7 +15510,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>41</t>
         </is>
@@ -15601,7 +15602,7 @@
           <t>90</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>26</t>
         </is>
@@ -15693,7 +15694,7 @@
           <t>127</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>36</t>
         </is>
@@ -15785,7 +15786,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -15877,7 +15878,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -15969,7 +15970,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -16061,7 +16062,7 @@
           <t>15</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -16153,7 +16154,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -16245,7 +16246,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -16337,7 +16338,7 @@
           <t>310</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>122</t>
         </is>
@@ -16533,7 +16534,7 @@
           <t>초등교육과</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -16630,7 +16631,7 @@
           <t>초등교육과</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr"/>
+      <c r="C21" s="8" t="inlineStr"/>
       <c r="D21" s="8" t="inlineStr">
         <is>
           <t>24</t>
@@ -16687,7 +16688,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr"/>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -16888,7 +16889,7 @@
           <t>초등교육과</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>90</t>
         </is>
@@ -16985,7 +16986,7 @@
           <t>초등교육과</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
+      <c r="C26" s="8" t="inlineStr"/>
       <c r="D26" s="8" t="inlineStr">
         <is>
           <t>19</t>
@@ -17042,7 +17043,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr"/>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>90</t>
         </is>
@@ -17243,7 +17244,7 @@
           <t>초등교육과</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>127</t>
         </is>
@@ -17340,7 +17341,7 @@
           <t>초등교육과</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr"/>
+      <c r="C31" s="8" t="inlineStr"/>
       <c r="D31" s="8" t="inlineStr">
         <is>
           <t>19</t>
@@ -17397,7 +17398,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr"/>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>127</t>
         </is>
@@ -17593,7 +17594,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -17685,7 +17686,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -17876,7 +17877,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -17968,7 +17969,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -18159,7 +18160,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -18251,7 +18252,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -18442,7 +18443,7 @@
           <t>15</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -18534,7 +18535,7 @@
           <t>15</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -18725,7 +18726,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -18817,7 +18818,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -19008,7 +19009,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -19100,7 +19101,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C56" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -19183,15 +19184,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19203,28 +19204,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19233,57 +19233,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -19399,7 +19400,7 @@
           <t>65</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>38</t>
         </is>
@@ -19491,7 +19492,7 @@
           <t>125</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>64</t>
         </is>
@@ -19583,7 +19584,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -19675,7 +19676,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -19767,7 +19768,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -19859,7 +19860,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -19951,7 +19952,7 @@
           <t>222</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>120</t>
         </is>
@@ -20034,15 +20035,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20054,28 +20055,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20084,57 +20084,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -20250,7 +20251,7 @@
           <t>133</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
+      <c r="C5" s="8" t="inlineStr"/>
       <c r="D5" s="8" t="inlineStr"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
@@ -20310,7 +20311,7 @@
           <t>57</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
+      <c r="C6" s="8" t="inlineStr"/>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
@@ -20370,7 +20371,7 @@
           <t>190</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
@@ -20421,15 +20422,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20441,28 +20442,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20471,57 +20471,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -20637,7 +20638,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>65</t>
         </is>
@@ -20729,7 +20730,7 @@
           <t>114</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>35</t>
         </is>
@@ -20821,7 +20822,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -20913,7 +20914,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -21005,7 +21006,7 @@
           <t>11</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -21097,7 +21098,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -21189,7 +21190,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -21281,7 +21282,7 @@
           <t>195</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>127</t>
         </is>
@@ -21364,15 +21365,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21384,28 +21385,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21414,57 +21414,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -21580,7 +21581,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>44</t>
         </is>
@@ -21672,7 +21673,7 @@
           <t>123</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>72</t>
         </is>
@@ -21764,7 +21765,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -21856,7 +21857,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -21948,7 +21949,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>30</t>
         </is>
@@ -22040,7 +22041,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -22132,7 +22133,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -22224,7 +22225,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -22316,7 +22317,7 @@
           <t>228</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>184</t>
         </is>
@@ -22507,7 +22508,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>44</t>
         </is>
@@ -22698,7 +22699,7 @@
           <t>123</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>72</t>
         </is>
@@ -22889,7 +22890,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -23080,7 +23081,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -23271,7 +23272,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>30</t>
         </is>
@@ -23462,7 +23463,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -23653,7 +23654,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -23844,7 +23845,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -23936,7 +23937,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -24019,15 +24020,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -24039,28 +24040,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:R12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -24069,57 +24069,58 @@
           <t>전체 경쟁률 현황</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>09월07일20시</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>09월08일20시</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>09월09일20시</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>09월10일20시</t>
         </is>
       </c>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>09월11일10시</t>
         </is>
       </c>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>09월11일14시</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>09월11일15시</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>최종</t>
         </is>
       </c>
-      <c r="S1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2027 수시모집 최종 경쟁률 마감 현황</t>
         </is>
@@ -24235,7 +24236,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>112</t>
         </is>
@@ -24327,7 +24328,7 @@
           <t>132</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>54</t>
         </is>
@@ -24419,7 +24420,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -24511,7 +24512,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -24603,7 +24604,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -24695,7 +24696,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -24787,7 +24788,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -24879,7 +24880,7 @@
           <t>209</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>212</t>
         </is>
@@ -24962,15 +24963,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>